<commit_message>
Add Product 3 images and update HTML structure for product details
</commit_message>
<xml_diff>
--- a/Assets/Product Catalog/catalog.xlsx
+++ b/Assets/Product Catalog/catalog.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -528,6 +528,34 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Portronics Snapcase 60W Multifunctional Cable Kit</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>299</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>60W fast-charging cable kit that adapts USB-A or Type-C to Micro-USB, Type-C, or Lightning. Compact ABS case with built-in SIM eject pin, spare SIM storage, mirror, and fold-out phone holder.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0DBR696V2?&amp;linkCode=ll2&amp;tag=viliwyth-21&amp;linkId=0d8c3df63041a60b842f7bbd5c17dff7&amp;ref_=as_li_ss_tl</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add pricing structure to product cards and modals
</commit_message>
<xml_diff>
--- a/Assets/Product Catalog/catalog.xlsx
+++ b/Assets/Product Catalog/catalog.xlsx
@@ -429,14 +429,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="90" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -458,15 +458,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>MRP</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Final Price</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Short Description</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Amazon Link</t>
         </is>
@@ -487,14 +492,17 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
+        <v>2999</v>
+      </c>
+      <c r="E2" s="2" t="n">
         <v>949</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>3-Tier vacuum-insulated stainless steel lunch jar — 900ml total, keeps food hot up to 6 hours, includes built-in spoon &amp; fork.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>https://www.amazon.in/YELONA-Insulated-Stainless-Leakproof-Dishwasher/dp/B0FMS3YN5Y?_encoding=UTF8&amp;pd_rd_w=5rJVW&amp;content-id=amzn1.sym.8742e3a6-fb96-4d77-a224-37a14c91ffb2&amp;pf_rd_p=8742e3a6-fb96-4d77-a224-37a14c91ffb2&amp;pf_rd_r=QZ7FPAYMJ0T3AY2VFE3G&amp;pd_rd_wg=YjTsp&amp;pd_rd_r=3677a84d-f82f-458c-b209-2485d5211468&amp;th=1&amp;linkCode=ll2&amp;tag=viliwyth-21&amp;linkId=f907df8c2d89d8f93801ee7f1d72c377&amp;ref_=as_li_ss_tl</t>
         </is>
@@ -515,14 +523,17 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
+        <v>999</v>
+      </c>
+      <c r="E3" s="2" t="n">
         <v>590</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>7L cabinet-door / wall-mounted plastic trash can with double-sided flip lid. Frees up floor space in tight kitchens; wipes clean easily.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0CFL39N3M?th=1&amp;linkCode=ll2&amp;tag=viliwyth-21&amp;linkId=598a20d185c908aafc69f863618868e3&amp;ref_=as_li_ss_tl</t>
         </is>
@@ -543,14 +554,17 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
+        <v>799</v>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>299</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>60W fast-charging cable kit that adapts USB-A or Type-C to Micro-USB, Type-C, or Lightning. Compact ABS case with built-in SIM eject pin, spare SIM storage, mirror, and fold-out phone holder.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>https://www.amazon.in/dp/B0DBR696V2?&amp;linkCode=ll2&amp;tag=viliwyth-21&amp;linkId=0d8c3df63041a60b842f7bbd5c17dff7&amp;ref_=as_li_ss_tl</t>
         </is>

</xml_diff>

<commit_message>
Add Product 4 images and details to the catalog and update styling for the carousel
</commit_message>
<xml_diff>
--- a/Assets/Product Catalog/catalog.xlsx
+++ b/Assets/Product Catalog/catalog.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -570,6 +570,37 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Home &amp; Kitchen</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Ember Cookware Silicone Flip Spatula (34 cm, Green)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>625</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>399</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>34 cm platinum-grade silicone flip spatula. Thin precision edge for dosa, pancakes &amp; cutlets. Seamless unibody, non-scratch on all cookware, dishwasher safe, heat-safe up to 230°C.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0GPKK2N3D?social_share=cm_sw_r_cso_wa_apin_dp_JWCKQKS4XVEQ81BJG2Q8&amp;th=1&amp;linkCode=ll2&amp;tag=viliwyth-21&amp;linkId=cffecb1c2d85186c45768d3238ce7f93&amp;ref_=as_li_ss_tl</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Product 5 and Product 6 details, images, and modals; update styling for Today's Picks section
</commit_message>
<xml_diff>
--- a/Assets/Product Catalog/catalog.xlsx
+++ b/Assets/Product Catalog/catalog.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -601,6 +601,68 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Portronics Clean G 20-in-1 Multipurpose Device Cleaning Kit</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1599</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>579</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Pocket-sized 20-in-1 cleaning kit for laptops, smartphones, keyboards, desktops &amp; earphones. Specialized brushes, microfiber pads and precision tips lift dust safely from screens, keys and ports.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0CG1WJVH3?th=1&amp;linkCode=ll2&amp;tag=viliwyth-21&amp;linkId=95afa7b4ef91a29fa107c188ed9df9f0&amp;ref_=as_li_ss_tl</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>JioTag Air Worldwide Tracker for iOS (Gray)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2999</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>749</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Bluetooth tracker that pairs with the Apple Find My app for worldwide locating of keys, luggage, bikes &amp; wallets. 120 dB buzzer for nearby finds, no SIM/subscription, ships with extra battery for ~2 years of use.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/dp/B0D59VZ1RS?th=1&amp;linkCode=ll2&amp;tag=viliwyth-21&amp;linkId=62d14b0631fa2cdc722c2af312581be1&amp;ref_=as_li_ss_tl</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>